<commit_message>
fix 2 file excel
</commit_message>
<xml_diff>
--- a/output/Laporan_Arah_Validasi_2025.xlsx
+++ b/output/Laporan_Arah_Validasi_2025.xlsx
@@ -474,16 +474,16 @@
         <v>45985.15302083334</v>
       </c>
       <c r="B2" t="n">
-        <v>-7.977602926040744</v>
+        <v>-7.986112910910143</v>
       </c>
       <c r="C2" t="n">
-        <v>113.4222419331524</v>
+        <v>113.4167560065577</v>
       </c>
       <c r="D2" t="n">
-        <v>246.5272061661201</v>
+        <v>246.8463597035008</v>
       </c>
       <c r="E2" t="n">
-        <v>191.9799470901489</v>
+        <v>194.298791885376</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -499,16 +499,16 @@
         <v>46049.34773148148</v>
       </c>
       <c r="B3" t="n">
-        <v>-7.977602926040744</v>
+        <v>-7.986112910910143</v>
       </c>
       <c r="C3" t="n">
-        <v>113.4222419331524</v>
+        <v>113.4167560065577</v>
       </c>
       <c r="D3" t="n">
-        <v>246.5272061661201</v>
+        <v>246.8463597035008</v>
       </c>
       <c r="E3" t="n">
-        <v>183.9334917068481</v>
+        <v>175.9845077991486</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>